<commit_message>
docs: add Build Log & Validation sheet with step-1 results and open gaps
Records measured step-1 outcomes (raw 80% coverage 79.2%, CQR 91.5%, MASE
TimesFM/ARIMA/naive 4.33/4.22/4.21, 0 headline breaches) and the goal
verification against the evaluation criteria, plus carried-forward gaps
(GARCH baseline, frozen holdout) so the design doc stays the source of truth.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tariff_Shock_EWS_Solution_Design.xlsx
+++ b/docs/Tariff_Shock_EWS_Solution_Design.xlsx
@@ -19,6 +19,7 @@
     <sheet name="8. File Structure" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="9. Evaluation &amp; Backtest" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="10. NFRs &amp; Risks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="11. Build Log &amp; Validation" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -177,7 +178,7 @@
       <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -247,6 +248,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009C6500"/>
       </patternFill>
     </fill>
   </fills>
@@ -418,7 +424,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -592,6 +598,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2247,6 +2259,598 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Build Log &amp; Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>What has actually been built and measured, versus the documented goals</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Build progression (against the file-structure build order)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Build order step</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>1. prices + forecaster</t>
+        </is>
+      </c>
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>Zero-shot forecast plotted</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E6" s="37" t="inlineStr">
+        <is>
+          <t>outputs/figures/*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="inlineStr">
+        <is>
+          <t>2. conformal + backtest</t>
+        </is>
+      </c>
+      <c r="B7" s="37" t="inlineStr">
+        <is>
+          <t>Calibrated intervals + coverage</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D7" s="37" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E7" s="37" t="inlineStr">
+        <is>
+          <t>step1_summary.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>3. events + attribution</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Event table + breach attribution</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="69" t="inlineStr">
+        <is>
+          <t>4. event eval</t>
+        </is>
+      </c>
+      <c r="B9" s="69" t="inlineStr">
+        <is>
+          <t>Lead-time / precision / attribution acc.</t>
+        </is>
+      </c>
+      <c r="C9" s="69" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="D9" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="69" t="inlineStr">
+        <is>
+          <t>after step 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="69" t="inlineStr">
+        <is>
+          <t>5. notebook + writeup</t>
+        </is>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>Shareable case study</t>
+        </is>
+      </c>
+      <c r="C10" s="69" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D10" s="69" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E10" s="69" t="inlineStr">
+        <is>
+          <t>README worked example</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Step-1 goal verification (forecast + calibration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Goal / eval criterion</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Target / pass bar</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Measured result</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>G1 Calibrated forecast</t>
+        </is>
+      </c>
+      <c r="B15" s="37" t="inlineStr">
+        <is>
+          <t>90% interval covers ~90%</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>91.5% coverage</t>
+        </is>
+      </c>
+      <c r="D15" s="37" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="E15" s="37" t="inlineStr">
+        <is>
+          <t>CQR offset Q=1.55 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>Interval calibration (headline)</t>
+        </is>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
+        <is>
+          <t>coverage ~ nominal</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>raw 80% -&gt; 79.2%; cal -&gt; 91.5%</t>
+        </is>
+      </c>
+      <c r="D16" s="37" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="E16" s="37" t="inlineStr">
+        <is>
+          <t>TimesFM deciles near-calibrated</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="69" t="inlineStr">
+        <is>
+          <t>Forecast quality (MASE)</t>
+        </is>
+      </c>
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>beat seasonal-naive</t>
+        </is>
+      </c>
+      <c r="C17" s="69" t="inlineStr">
+        <is>
+          <t>TimesFM 4.33 vs naive 4.21</t>
+        </is>
+      </c>
+      <c r="D17" s="69" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E17" s="69" t="inlineStr">
+        <is>
+          <t>Explained: efficient ETF ~ random walk</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="69" t="inlineStr">
+        <is>
+          <t>Baseline gauntlet</t>
+        </is>
+      </c>
+      <c r="B18" s="69" t="inlineStr">
+        <is>
+          <t>naive / ARIMA / GARCH</t>
+        </is>
+      </c>
+      <c r="C18" s="69" t="inlineStr">
+        <is>
+          <t>naive + ARIMA done</t>
+        </is>
+      </c>
+      <c r="D18" s="69" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E18" s="69" t="inlineStr">
+        <is>
+          <t>GARCH not yet implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="69" t="inlineStr">
+        <is>
+          <t>Robustness</t>
+        </is>
+      </c>
+      <c r="B19" s="69" t="inlineStr">
+        <is>
+          <t>frozen ~6-month holdout</t>
+        </is>
+      </c>
+      <c r="C19" s="69" t="inlineStr">
+        <is>
+          <t>rolling origins + 10d holdout</t>
+        </is>
+      </c>
+      <c r="D19" s="69" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="E19" s="69" t="inlineStr">
+        <is>
+          <t>Frozen holdout still to add</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="37" t="inlineStr">
+        <is>
+          <t>G4 Checkable</t>
+        </is>
+      </c>
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>dated, falsifiable, reproducible</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
+        <is>
+          <t>dated example + script</t>
+        </is>
+      </c>
+      <c r="D20" s="37" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="E20" s="37" t="inlineStr">
+        <is>
+          <t>step1_forecast_slx.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Step-1 measured results (SLX, 2016-01-04 to 2026-07-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="17" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Backbone / calibration</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>TimesFM 2.5 zero-shot + split-conformal CQR</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Horizon</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>10 business days</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="20" t="n"/>
+      <c r="E26" s="20" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Raw q10-q90 coverage (nominal 80%)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>79.2%</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>CQR-calibrated coverage (target 90%)</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>91.5%</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="20" t="n"/>
+      <c r="E28" s="20" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>CQR offset Q</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>1.55 (USD)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>MASE  TimesFM / ARIMA / naive</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>4.33 / 4.22 / 4.21</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="20" t="n"/>
+      <c r="E30" s="20" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>Headline holdout (2026-06-24 -&gt; 07-08)</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>0 interval breaches</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="70" t="inlineStr">
+        <is>
+          <t>Open gaps carried forward (do not drift, close these)</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>•  GARCH volatility baseline: add to the gauntlet alongside ARIMA + seasonal-naive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>•  Frozen ~6-month holdout: implement the untouched holdout the design specifies for robustness.</t>
+        </is>
+      </c>
+      <c r="B36" s="36" t="n"/>
+      <c r="C36" s="36" t="n"/>
+      <c r="D36" s="36" t="n"/>
+      <c r="E36" s="36" t="n"/>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>•  Point accuracy vs naive: expected to improve on less-efficient targets (HRC futures, freight rates), not broad ETFs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>•  Event layer (G2/G3): build-step 3 wires the Federal Register events + breach monitor + attribution.</t>
+        </is>
+      </c>
+      <c r="B38" s="36" t="n"/>
+      <c r="C38" s="36" t="n"/>
+      <c r="D38" s="36" t="n"/>
+      <c r="E38" s="36" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="B28:E28"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
docs: log v2 plan (sheet 12) - workstreams, backbone decision, acceptance criteria
Design doc rev 1.3 / 'v2 In Progress'. New sheet '12. v2 Plan & Progress':
- W1 covariate-aware forecasting: TimesFM 2.5 XReg first (proven backbone kept),
  Moirai-2 explicitly demoted to fallback; covariate set pre-registered
  (UUP, CL=F, HG=F; carry-forward persistence for the horizon, no lookahead);
  primary metric = mean ACI-calibrated width at matched 90% coverage
- W2 aluminum vertical via config only (extensibility NFR proof)
- W3 machine-readable alert artifacts + inert webhook stub
- v2 evaluation principles carried from v1 (pre-registration, identical arms,
  publish nulls, document before Done)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tariff_Shock_EWS_Solution_Design.xlsx
+++ b/docs/Tariff_Shock_EWS_Solution_Design.xlsx
@@ -20,6 +20,7 @@
     <sheet name="9. Evaluation &amp; Backtest" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="10. NFRs &amp; Risks" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="11. Build Log &amp; Validation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="12. v2 Plan &amp; Progress" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,7 +425,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -613,6 +614,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1105,7 +1112,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>1.2 (v1 delivered)</t>
+          <t>1.3 (v2 in progress)</t>
         </is>
       </c>
       <c r="D16" s="8" t="n"/>
@@ -1120,7 +1127,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>v1 complete: pipeline live, all logged gaps closed with evidence</t>
+          <t>v1 complete and live; v2 workstreams W1-W3 planned on sheet 12</t>
         </is>
       </c>
       <c r="D17" s="8" t="n"/>
@@ -3358,13 +3365,218 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>v2 Plan &amp; Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Workstreams, decisions, and pre-registered acceptance criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Workstreams</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Workstream</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Acceptance criteria (pre-registered)</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66" customHeight="1">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>W1. Covariate-aware forecasting</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Exogenous covariates via TimesFM 2.5 XReg (forecast_with_covariates, timesfm[xreg]). Covariate set fixed upfront: UUP (USD), CL=F (oil), HG=F (copper), all yfinance daily, no key. Future covariate values = carry-forward persistence (no lookahead).</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>PRIMARY: mean ACI-calibrated interval width at matched 90% coverage, XReg arm vs v1 cached arm on identical HRC rolling origins. SECONDARY: MASE. XReg ships only if it improves the primary without degrading coverage; else v1 stands and Moirai-2 is evaluated.</t>
+        </is>
+      </c>
+      <c r="D6" s="66" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>W2. Aluminum vertical</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>config/aluminum.yaml only (Section 232 also covers aluminum); zero code changes.</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>python -m src.pipeline --config config/aluminum.yaml runs end-to-end and produces a band-history cache + alert scan. Proves the extensibility NFR.</t>
+        </is>
+      </c>
+      <c r="D7" s="67" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>W3. Alert delivery</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Pipeline writes machine-readable alert artifacts to outputs/alerts/&lt;vertical&gt;_&lt;date&gt;.json; optional webhook URL in config (stub, off by default).</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Artifact produced on a real run; schema documented; webhook config present but inert unless set.</t>
+        </is>
+      </c>
+      <c r="D8" s="67" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>W1 backbone decision (supersedes the v1-era 'Moirai-2 for v2' note)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="74" t="inlineStr">
+        <is>
+          <t>DECISION: attempt covariates with TimesFM 2.5 XReg FIRST, keeping the proven v1 backbone, ACI calibration, and pipeline unchanged (one optional dependency: timesfm[xreg]). Moirai-2 remains the fallback, evaluated only if XReg fails to run or does not improve the pre-registered primary metric. Rationale: incremental risk, directly comparable arms on the same cached rolling origins, and no re-validation of the calibration stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="17">
+      <c r="A17" s="75" t="inlineStr">
+        <is>
+          <t>v2 evaluation principles (carried from v1)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>•  Every claim pre-registered before results are seen; nulls are published, not buried.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>•  Arms compared on identical rolling origins with the same ACI settings (gamma=0.02, warmup=50).</t>
+        </is>
+      </c>
+      <c r="B19" s="36" t="n"/>
+      <c r="C19" s="36" t="n"/>
+      <c r="D19" s="36" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>•  No lookahead: future covariate values are carry-forward persistence, never realized futures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>•  Results land in this sheet + README + a step JSON before any status flips to Done.</t>
+        </is>
+      </c>
+      <c r="B21" s="36" t="n"/>
+      <c r="C21" s="36" t="n"/>
+      <c r="D21" s="36" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A12:D15"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A19:D19"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3527,310 +3739,332 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>v2 plan logged (sheet 12): W1 covariates via TimesFM XReg (Moirai-2 fallback), W2 aluminum vertical config-only, W3 alert delivery; W1 eval pre-registered</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>v2 In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Approvals</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>Responsibility</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Sign-off</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Design Authority</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>(owner)</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Overall design sign-off</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Data / ML Lead</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>(TBD)</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>Model + data feasibility</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Risk Stakeholder</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>(TBD)</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Business value &amp; metrics</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Glossary</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Definition</t>
         </is>
       </c>
-      <c r="C21" s="16" t="n"/>
-      <c r="D21" s="16" t="n"/>
-      <c r="E21" s="17" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="17" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>Zero-shot</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>Forecasting a new series with a pretrained model, no per-series retraining.</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Foundation model</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Large pretrained time-series model (Chronos-2, TimesFM, Moirai-2).</t>
         </is>
       </c>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="20" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="C24" s="20" t="n"/>
+      <c r="D24" s="20" t="n"/>
+      <c r="E24" s="20" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>Conformal prediction</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>Wrapper giving prediction intervals with empirically guaranteed coverage.</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>CQR</t>
         </is>
       </c>
-      <c r="B25" s="15" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Conformalized Quantile Regression; offsets a model's q10/q90 band to hit target coverage.</t>
         </is>
       </c>
-      <c r="C25" s="20" t="n"/>
-      <c r="D25" s="20" t="n"/>
-      <c r="E25" s="20" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="20" t="n"/>
+      <c r="E26" s="20" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>TimesFM 2.5</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>Google's 200M-param decoder-only time-series foundation model; zero-shot, quantile head.</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="8" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Fraction of actuals that fall inside the predicted interval (should match nominal, e.g. 90%).</t>
         </is>
       </c>
-      <c r="C27" s="20" t="n"/>
-      <c r="D27" s="20" t="n"/>
-      <c r="E27" s="20" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="20" t="n"/>
+      <c r="E28" s="20" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>Interval breach</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Actual value falls outside the calibrated forecast interval -&gt; candidate shock.</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="8" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>Changepoint</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Statistically detected structural break in a series (via PELT / BOCPD).</t>
         </is>
       </c>
-      <c r="C29" s="20" t="n"/>
-      <c r="D29" s="20" t="n"/>
-      <c r="E29" s="20" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="20" t="n"/>
+      <c r="E30" s="20" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Attribution</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>Ranking candidate events to name the most likely driver of a break.</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="n"/>
-      <c r="E30" s="8" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>EWS</t>
         </is>
       </c>
-      <c r="B31" s="15" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>Early-Warning System.</t>
         </is>
       </c>
-      <c r="C31" s="20" t="n"/>
-      <c r="D31" s="20" t="n"/>
-      <c r="E31" s="20" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="20" t="n"/>
+      <c r="E32" s="20" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>MASE</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>Mean Absolute Scaled Error; scale-free forecast accuracy vs seasonal-naive.</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="8" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>FBX</t>
         </is>
       </c>
-      <c r="B33" s="15" t="inlineStr">
+      <c r="B34" s="15" t="inlineStr">
         <is>
           <t>Freightos Baltic Index (container shipping cost).</t>
         </is>
       </c>
-      <c r="C33" s="20" t="n"/>
-      <c r="D33" s="20" t="n"/>
-      <c r="E33" s="20" t="n"/>
+      <c r="C34" s="20" t="n"/>
+      <c r="D34" s="20" t="n"/>
+      <c r="E34" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -3839,13 +4073,13 @@
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="B21:E21"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B34:E34"/>
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="B22:E22"/>
     <mergeCell ref="B32:E32"/>

</xml_diff>

<commit_message>
docs: post-v2 gap register (sheet 12) - 5 gaps from the close-out audit
G1 no automated tests for core quant logic; G2 aluminum calibration unvalidated
(runs != calibrated); G3 ACI gamma=0.02 an untested default; G4 band cache lacks
a config guard (silent corruption on horizon/symbol change); G5 no scheduled
execution. Each logged with risk-if-open and the planned fix; to be closed in
order with per-gap commits.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tariff_Shock_EWS_Solution_Design.xlsx
+++ b/docs/Tariff_Shock_EWS_Solution_Design.xlsx
@@ -3422,7 +3422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3683,14 +3683,157 @@
       <c r="C28" s="36" t="n"/>
       <c r="D28" s="36" t="n"/>
     </row>
+    <row r="30">
+      <c r="A30" s="73" t="inlineStr">
+        <is>
+          <t>Post-v2 gap register (found in the v2 close-out audit; solve in order)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Risk if left open</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="52" customHeight="1">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>G1. No automated tests for core quant logic</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Regressions in CQR/ACI math, severity rules, attribution ranking, or the alert schema ship silently; all verification so far was manual</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>pytest suite: synthetic coverage-guarantee tests for cqr_offset/aci_cqr, rule tests for severity, stub-embedder tests for attribution, schema test for deliver()</t>
+        </is>
+      </c>
+      <c r="D32" s="66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="52" customHeight="1">
+      <c r="A33" s="41" t="inlineStr">
+        <is>
+          <t>G2. Aluminum calibration unvalidated</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>W2 proved the pipeline RUNS on ALI=F, not that ACI holds ~90% coverage there; alerts on an uncalibrated vertical are untrustworthy</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Run ACI over the cached bands_aluminum.parquet; record realized coverage here</t>
+        </is>
+      </c>
+      <c r="D33" s="66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="52" customHeight="1">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>G3. ACI gamma=0.02 is an untested default</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>A lucky constant: calibration quality could hinge on one literature value never checked on our series</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Sweep gamma in {0.005, 0.01, 0.02, 0.05, 0.1} on cached HRC + SLX bands. Pre-registered: keep 0.02 unless another value clearly dominates |coverage-90| on BOTH series</t>
+        </is>
+      </c>
+      <c r="D34" s="66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="52" customHeight="1">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
+          <t>G4. Band cache lacks a config guard</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Changing horizon_days or the target symbol silently feeds stale cached bands into ACI (wrong intervals, no error)</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Sidecar meta (symbol, horizon, quantiles) written with the cache; mismatch invalidates and recomputes; unit test</t>
+        </is>
+      </c>
+      <c r="D35" s="66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="52" customHeight="1">
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>G5. No scheduled execution</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>The 'daily batch' only runs when someone remembers; stale alerts read as 'all clear'</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>scripts/run_daily.bat for both verticals + README ops note with the Windows Task Scheduler registration command</t>
+        </is>
+      </c>
+      <c r="D36" s="66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A30:D30"/>
     <mergeCell ref="A12:D15"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A24:D24"/>

</xml_diff>

<commit_message>
Close post-v2 gap G1: pytest suite for core quantitative logic (25 tests)
Network-free, deterministic (seeded), no model downloads:
- conformal: CQR reaches target coverage from too-narrow AND too-wide bands
  (negative offsets), empty-input safety, multi-target parametrization; ACI
  holds ~90% on stationary noise and through a 2.5x variance regime shift
- events: severity rules (Section 232, proclamation language, cap, vectorized),
  attribution ranking with a stub embedder (recency/relevance ordering,
  lookback/future exclusion, top-k, and the object-dtype published regression)
- eval + delivery: lead-time/precision-recall/attribution-accuracy metrics;
  alert artifact schema incl. zero-alert runs and webhook-failure isolation

pyproject: [tool.pytest.ini_options] pythonpath/testpaths. Run: pytest -q.
docs/: gap register G1 -> Closed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tariff_Shock_EWS_Solution_Design.xlsx
+++ b/docs/Tariff_Shock_EWS_Solution_Design.xlsx
@@ -3728,12 +3728,12 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>pytest suite: synthetic coverage-guarantee tests for cqr_offset/aci_cqr, rule tests for severity, stub-embedder tests for attribution, schema test for deliver()</t>
-        </is>
-      </c>
-      <c r="D32" s="66" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>pytest suite: synthetic coverage-guarantee tests for cqr_offset/aci_cqr (incl. regime-shift adaptation + negative-offset tightening), rule tests for severity, stub-embedder tests for attribution (incl. the object-dtype regression), event_eval metrics, deliver() schema + webhook-failure isolation. 25 tests green, network-free.</t>
+        </is>
+      </c>
+      <c r="D32" s="74" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close post-v2 gap G2: aluminum calibration validated (89.6% vs 90% target)
ACI over the pipeline's own cached ALI=F band history (600 days, 2024-03 to
2026-07): realized coverage 89.6% post-warmup (550 days, 57 breach-days),
mean calibrated width 300.7 USD/ton. Verdict: calibrated. Small-sample caveat
recorded; every alert continues to carry the realized coverage for monitoring.

docs/: gap register G2 -> Closed with the measured numbers.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tariff_Shock_EWS_Solution_Design.xlsx
+++ b/docs/Tariff_Shock_EWS_Solution_Design.xlsx
@@ -3750,12 +3750,12 @@
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t>Run ACI over the cached bands_aluminum.parquet; record realized coverage here</t>
-        </is>
-      </c>
-      <c r="D33" s="66" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Validated (step9): ACI realized coverage 89.6% vs 90% target over 550 post-warmup days (2024-03..2026-07), 57 breach-days, mean calibrated width 300.7 USD/ton. Small-sample caveat noted; coverage continues to be monitored on every alert.</t>
+        </is>
+      </c>
+      <c r="D33" s="74" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close post-v2 gap G3: ACI gamma sweep - 0.02 kept, default is robust
Sweep over {0.005, 0.01, 0.02, 0.05, 0.1} on both cached band histories
(2110 days each, no model calls). Coverage stays within ~0.5pp of the 90%
target across 0.005-0.05 on both HRC=F and SLX; only 0.1 degrades (>1pp).
Per the pre-registered rule (challenger must dominate by >=1pp on BOTH
series), gamma=0.02 is kept. Width falls monotonically with gamma, as
expected (faster adaptation = tighter but riskier), reported as context.

docs/: gap register G3 -> Closed with the sweep numbers.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tariff_Shock_EWS_Solution_Design.xlsx
+++ b/docs/Tariff_Shock_EWS_Solution_Design.xlsx
@@ -3772,12 +3772,12 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>Sweep gamma in {0.005, 0.01, 0.02, 0.05, 0.1} on cached HRC + SLX bands. Pre-registered: keep 0.02 unless another value clearly dominates |coverage-90| on BOTH series</t>
-        </is>
-      </c>
-      <c r="D34" s="66" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Swept (step10): coverage within ~0.5pp of target for gamma 0.005-0.05 on BOTH series (HRC 89.6-90.2%, SLX 89.2-89.7%); only gamma=0.1 degrades (&gt;1pp). No challenger dominates; 0.02 KEPT per the pre-registered rule. The default is robust, not lucky.</t>
+        </is>
+      </c>
+      <c r="D34" s="74" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close post-v2 gap G4: band-cache config guard
A band cache built under a different symbol/horizon/quantile config could
silently corrupt ACI's input. _band_history now writes a sidecar
bands_<vertical>.meta.json and invalidates (recomputes with a printed notice)
on any mismatch or missing meta. Pre-guard caches recompute once by design.

4 unit tests with a stub forecaster (no model): full cache hit skips
recompute; horizon change, symbol change, and missing meta all invalidate.
Suite: 29 passed.

docs/: gap register G4 -> Closed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tariff_Shock_EWS_Solution_Design.xlsx
+++ b/docs/Tariff_Shock_EWS_Solution_Design.xlsx
@@ -3794,12 +3794,12 @@
       </c>
       <c r="C35" s="14" t="inlineStr">
         <is>
-          <t>Sidecar meta (symbol, horizon, quantiles) written with the cache; mismatch invalidates and recomputes; unit test</t>
-        </is>
-      </c>
-      <c r="D35" s="66" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Implemented: sidecar bands_&lt;vertical&gt;.meta.json (symbol, horizon, quantiles) written with the cache; mismatch or missing meta invalidates and recomputes with a printed notice. 4 unit tests (hit, horizon change, symbol change, pre-guard cache). One-time recompute of existing caches.</t>
+        </is>
+      </c>
+      <c r="D35" s="74" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close post-v2 gap G5: scheduled daily batch + ops runbook (register complete)
scripts/run_daily.bat runs every vertical with per-vertical logs
(outputs/logs/, gitignored) and delayed expansion for correct timestamps;
README Operations section documents the Windows Task Scheduler registration.
Missing daily artifact now means 'did not run', never 'all clear'.

Verified end-to-end on both verticals. The run also regenerated both band
caches under the G4 meta guard, and produced the system's FIRST organic
production alert: aluminum 2026-07-10, ALI=F 3303.50 below the calibrated
floor 3331.76, with BOTH cross-checks agreeing (changepoint + GARCH) and an
honest empty candidate-driver list. Artifact committed as a live example.

docs/: gap register G5 -> Closed; file tree updated (tests/, step9, step10,
run_daily.bat). Post-v2 register: all 5 gaps closed. Suite: 29 passed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tariff_Shock_EWS_Solution_Design.xlsx
+++ b/docs/Tariff_Shock_EWS_Solution_Design.xlsx
@@ -1258,7 +1258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1654,223 +1654,271 @@
     <row r="35">
       <c r="A35" s="60" t="inlineStr">
         <is>
+          <t>├─ tests/</t>
+        </is>
+      </c>
+      <c r="B35" s="61" t="inlineStr">
+        <is>
+          <t>pytest suite: conformal math, events, eval, delivery, cache guard (G1/G4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="60" t="inlineStr">
+        <is>
           <t>├─ tools/</t>
         </is>
       </c>
-      <c r="B35" s="61" t="inlineStr">
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t>Repo meta-tooling</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="62" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="64" t="inlineStr">
         <is>
           <t>│   └─ build_design_doc.py</t>
         </is>
       </c>
-      <c r="B36" s="63" t="inlineStr">
+      <c r="B37" s="65" t="inlineStr">
         <is>
           <t>Regenerates docs/ solution design workbook</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="60" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="60" t="inlineStr">
         <is>
           <t>├─ scripts/</t>
         </is>
       </c>
-      <c r="B37" s="61" t="inlineStr">
+      <c r="B38" s="61" t="inlineStr">
         <is>
           <t>Runnable build-step scripts</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="62" t="inlineStr">
-        <is>
-          <t>│   ├─ step1_forecast_slx.py</t>
-        </is>
-      </c>
-      <c r="B38" s="63" t="inlineStr">
-        <is>
-          <t>Step 1: SLX TimesFM forecast + CQR interval + baselines</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="64" t="inlineStr">
         <is>
-          <t>│   ├─ step2_events_attribution.py</t>
+          <t>│   ├─ step1_forecast_slx.py</t>
         </is>
       </c>
       <c r="B39" s="65" t="inlineStr">
         <is>
-          <t>Step 2: breach detection + Federal Register attribution</t>
+          <t>Step 1: SLX TimesFM forecast + CQR interval + baselines</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="62" t="inlineStr">
         <is>
-          <t>│   ├─ step3_close_gaps.py</t>
+          <t>│   ├─ step2_events_attribution.py</t>
         </is>
       </c>
       <c r="B40" s="63" t="inlineStr">
         <is>
-          <t>Step 3: ACI, GARCH baseline, frozen holdout, permutation test</t>
+          <t>Step 2: breach detection + Federal Register attribution</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="64" t="inlineStr">
         <is>
-          <t>│   ├─ step4_hrc_attribution.py</t>
+          <t>│   ├─ step3_close_gaps.py</t>
         </is>
       </c>
       <c r="B41" s="65" t="inlineStr">
         <is>
-          <t>Step 4: pre-registered attribution retest on HRC futures</t>
+          <t>Step 3: ACI, GARCH baseline, frozen holdout, permutation test</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="62" t="inlineStr">
         <is>
-          <t>│   ├─ step5_forward_eval.py</t>
+          <t>│   ├─ step4_hrc_attribution.py</t>
         </is>
       </c>
       <c r="B42" s="63" t="inlineStr">
         <is>
-          <t>Step 5: forward early-warning eval (G3), ACI flags vs shocks</t>
+          <t>Step 4: pre-registered attribution retest on HRC futures</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="64" t="inlineStr">
         <is>
-          <t>│   ├─ step6_announcement_attribution.py</t>
+          <t>│   ├─ step5_forward_eval.py</t>
         </is>
       </c>
       <c r="B43" s="65" t="inlineStr">
         <is>
-          <t>Step 6: announcement-dated (TPU) attribution retest</t>
+          <t>Step 5: forward early-warning eval (G3), ACI flags vs shocks</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="62" t="inlineStr">
         <is>
-          <t>│   ├─ step7_alert_precision.py</t>
+          <t>│   ├─ step6_announcement_attribution.py</t>
         </is>
       </c>
       <c r="B44" s="63" t="inlineStr">
         <is>
-          <t>Step 7: pre-specified alert-precision filter evaluation</t>
+          <t>Step 6: announcement-dated (TPU) attribution retest</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="64" t="inlineStr">
         <is>
-          <t>│   └─ step8_covariates_eval.py</t>
+          <t>│   ├─ step7_alert_precision.py</t>
         </is>
       </c>
       <c r="B45" s="65" t="inlineStr">
         <is>
+          <t>Step 7: pre-specified alert-precision filter evaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="62" t="inlineStr">
+        <is>
+          <t>│   ├─ step8_covariates_eval.py</t>
+        </is>
+      </c>
+      <c r="B46" s="63" t="inlineStr">
+        <is>
           <t>Step 8 (v2-W1): XReg vs v1 pre-registered eval</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="60" t="inlineStr">
-        <is>
-          <t>├─ data/</t>
-        </is>
-      </c>
-      <c r="B46" s="61" t="inlineStr">
-        <is>
-          <t>Gitignored raw + parquet cache</t>
-        </is>
-      </c>
-    </row>
     <row r="47">
-      <c r="A47" s="60" t="inlineStr">
-        <is>
-          <t>└─ outputs/</t>
-        </is>
-      </c>
-      <c r="B47" s="61" t="inlineStr">
-        <is>
-          <t>Generated artifacts</t>
+      <c r="A47" s="64" t="inlineStr">
+        <is>
+          <t>│   ├─ step9_aluminum_validation.py</t>
+        </is>
+      </c>
+      <c r="B47" s="65" t="inlineStr">
+        <is>
+          <t>Step 9 (G2): aluminum ACI coverage validation</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ figures/</t>
+          <t>│   ├─ step10_gamma_sweep.py</t>
         </is>
       </c>
       <c r="B48" s="63" t="inlineStr">
         <is>
-          <t>Interval-breach plots for the writeup</t>
+          <t>Step 10 (G3): ACI gamma sensitivity sweep</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="64" t="inlineStr">
         <is>
+          <t>│   └─ run_daily.bat</t>
+        </is>
+      </c>
+      <c r="B49" s="65" t="inlineStr">
+        <is>
+          <t>Daily batch for all verticals + logs (G5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="60" t="inlineStr">
+        <is>
+          <t>├─ data/</t>
+        </is>
+      </c>
+      <c r="B50" s="61" t="inlineStr">
+        <is>
+          <t>Gitignored raw + parquet cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="60" t="inlineStr">
+        <is>
+          <t>└─ outputs/</t>
+        </is>
+      </c>
+      <c r="B51" s="61" t="inlineStr">
+        <is>
+          <t>Generated artifacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ figures/</t>
+        </is>
+      </c>
+      <c r="B52" s="63" t="inlineStr">
+        <is>
+          <t>Interval-breach plots for the writeup</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="64" t="inlineStr">
+        <is>
           <t xml:space="preserve">    └─ alerts/</t>
         </is>
       </c>
-      <c r="B49" s="65" t="inlineStr">
+      <c r="B53" s="65" t="inlineStr">
         <is>
           <t>Machine-readable alert artifacts per vertical/date (v2-W3)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>Recommended build order (always keep something working)</t>
         </is>
       </c>
-      <c r="B51" s="2" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="64" t="inlineStr">
-        <is>
-          <t>1. data/prices.py + forecast/chronos_model.py  -&gt;  a zero-shot forecast plotted (Day 1-2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="62" t="inlineStr">
-        <is>
-          <t>2. forecast/conformal.py + eval/backtest.py     -&gt;  calibrated intervals + coverage (Day 3-4)</t>
-        </is>
-      </c>
-      <c r="B53" s="36" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="64" t="inlineStr">
-        <is>
-          <t>3. data/events.py + events/*                     -&gt;  event table + attribution (Day 5-7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="62" t="inlineStr">
-        <is>
-          <t>4. eval/event_eval.py on real 2025-26 events     -&gt;  the money chart (Day 8-9)</t>
-        </is>
-      </c>
-      <c r="B55" s="36" t="n"/>
+      <c r="B55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="64" t="inlineStr">
+        <is>
+          <t>1. data/prices.py + forecast/chronos_model.py  -&gt;  a zero-shot forecast plotted (Day 1-2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="62" t="inlineStr">
+        <is>
+          <t>2. forecast/conformal.py + eval/backtest.py     -&gt;  calibrated intervals + coverage (Day 3-4)</t>
+        </is>
+      </c>
+      <c r="B57" s="36" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="64" t="inlineStr">
+        <is>
+          <t>3. data/events.py + events/*                     -&gt;  event table + attribution (Day 5-7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="62" t="inlineStr">
+        <is>
+          <t>4. eval/event_eval.py on real 2025-26 events     -&gt;  the money chart (Day 8-9)</t>
+        </is>
+      </c>
+      <c r="B59" s="36" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="64" t="inlineStr">
         <is>
           <t>5. notebooks/01 + README case study             -&gt;  the shareable artifact (Day 10)</t>
         </is>
@@ -1879,12 +1927,12 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A60:B60"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -3816,12 +3864,12 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>scripts/run_daily.bat for both verticals + README ops note with the Windows Task Scheduler registration command</t>
-        </is>
-      </c>
-      <c r="D36" s="66" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Implemented: scripts/run_daily.bat runs every vertical with per-vertical logs (outputs/logs/); README Operations section documents the schtasks registration. Verified end-to-end on both verticals; missing daily artifact now means 'did not run', never 'all clear'.</t>
+        </is>
+      </c>
+      <c r="D36" s="74" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>